<commit_message>
Paranda: lõikekadu arvutus ja lamellide profiili lahtilõike laius
- Lõikekadu: 696,839446 × 1,05 = 731,681 m² (mitte 733,515)
- Komposiitplaadid: 146 tk (eeldus plaadi laius 1200 mm)
- Lamellid: 1822,5 jm - tellimiskogus sõltub profiili lahtilõike
  laiusest koos pöördetega (andmed puuduvad)
- Märgitud selgelt: plaadi laius on eeldus, lamellide osa nõuab
  täiendavat profiili andmeid

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VioFG8PWR6ktkCEhY1HBJj
</commit_message>
<xml_diff>
--- a/Asula_14_plaadikulu.xlsx
+++ b/Asula_14_plaadikulu.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +64,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D9E8F5"/>
         <bgColor rgb="00D9E8F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -93,12 +109,15 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -467,10 +486,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -599,7 +618,7 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>36.67576031578947</v>
+        <v>34.8419723</v>
       </c>
     </row>
     <row r="16">
@@ -609,16 +628,16 @@
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>733.5152063157894</v>
+        <v>731.6814183</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Plaadi mõõdud (näide)</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+          <t>Plaadi mõõdud (EELDUS)</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>4200 mm × 1200 mm</t>
         </is>
@@ -630,7 +649,7 @@
           <t>Plaadi pind</t>
         </is>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="10" t="n">
         <v>5.04</v>
       </c>
     </row>
@@ -652,144 +671,157 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Lamellide tüüp</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Kogus (tk)</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Pikkus (m)</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Kogupikkus (jm)</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
-        <is>
-          <t>Profiiliga laius (mm)</t>
-        </is>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>Kogupind (m²)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Seinalamellid</t>
         </is>
       </c>
-      <c r="B26" s="11" t="n">
+      <c r="B26" s="12" t="n">
         <v>290</v>
       </c>
-      <c r="C26" s="11" t="n">
+      <c r="C26" s="12" t="n">
         <v>4.5</v>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D26" s="12" t="n">
         <v>1305</v>
       </c>
-      <c r="E26" s="11" t="n">
-        <v>205</v>
-      </c>
-      <c r="F26" s="4" t="n">
+      <c r="E26" s="4" t="n">
         <v>267.96</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Rõdulamellid</t>
         </is>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="12" t="n">
         <v>115</v>
       </c>
-      <c r="C27" s="11" t="n">
+      <c r="C27" s="12" t="n">
         <v>4.5</v>
       </c>
-      <c r="D27" s="11" t="n">
+      <c r="D27" s="12" t="n">
         <v>517.5</v>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>205</v>
-      </c>
-      <c r="F27" s="4" t="n">
+      <c r="E27" s="4" t="n">
         <v>106.26</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>KOKKU lamellid</t>
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>KOKKU lamellid (pikkus)</t>
         </is>
       </c>
       <c r="D28" s="5" t="n">
         <v>1822.5</v>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="E28" s="8" t="n">
         <v>374.22</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>LAMELLIDE PROFIILI LAHTILÕIKE LAIUS</t>
+        </is>
+      </c>
+    </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Profiili lahtilõike laius (mm)</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>PUUDUB - KÜSI KASUTAJALT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Lamellide ühikupikkus</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Oleneb profiilil - lamellide tellimiskogust ei saa määrata</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>MÄRKUSED</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="13" t="inlineStr">
-        <is>
-          <t>• Plaadi pikkus on 4200 mm, lamellide pikkus 4500 mm. Lamellide liited või pikemad plaadid on eraldi kokkuleppel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="13" t="inlineStr">
-        <is>
-          <t>• Plaadi laiuseks on eeldatud 1200 mm (5.04 m² plaat). Tegeliku laiuse korral korrektsioon vajalik.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
-        <is>
-          <t>• Lamellide profiiliga laius ~205 mm (0.924 m² per 4.5 m lamell).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>• Lõikekada arvestatud 5%.</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
-        <is>
-          <t>• Seina- ja rõdulamellid: sama profiil 205 mm laiusega.</t>
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>• Plaadi laiuseks eeldatud 1200 mm (standard). Kui laius erineb, korrektsioon vajalik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>• Plaadi pikkus on 4200 mm, lamellide pikkus 4500 mm. Lamellide liited või pikemad plaadid kokkuleppel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>• Lamellide materjalikulu (tellimiskogus) sõltub profiili lahtilõike laiusest koos pöördetega.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>• Kuni profiili lahtilõike laius teada pole, lamellide lõplik tellimiskogus määrata ei saa.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A34:E34"/>
-    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A38:E38"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="B32:C32"/>
     <mergeCell ref="A36:E36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>